<commit_message>
Modified excel files after running the script
</commit_message>
<xml_diff>
--- a/wildberries_filtered_catalog.xlsx
+++ b/wildberries_filtered_catalog.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,62 +486,604 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.wildberries.ru/catalog/239833866/detail.aspx</t>
+          <t>https://www.wildberries.ru/catalog/277883751/detail.aspx</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>239833866</v>
+        <v>277883751</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Полупальто шерстяное</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>8030</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Серое полупальто женское французского бренда Maison David. Состав: 100% шерсть натуральная. Шерсть отлично согревает, при этом позволяет телу дышать, не создавая парникового эффекта. В шерстяных вещах тепло, но не жарко. Одежда из шерсти — идеальный выбор для зимы и холодного демисезона. Состав подкладки: полиэстер, вискоза.
+Верхняя одежда имеет прямой силуэт. Модель отличает отложной воротник и наличие прорезных карманов. Температурный режим от плюс 10 до минус 5.
+Ухаживайте за вещью правильно, чтобы она дольше служила и радовала вас. Правила по уходу указаны на вшивном ярлычке изделия. Разрешено: химчистка. Запрещено: стирка, отбеливание, глажка, барабанная сушка.
+Полупальто в деловом стиле — удачное решение для офисного гардероба. Это сдержанная элегантность, уверенность и профессионализм. Maison David — дом современной элегантности. Бренд отражает идею французского bon chic, bon genre: искусство быть безупречным без усилий, сочетая гармонию интеллекта и формы, а качество становится главным языком красоты. Бренд соединяет современные тенденции с классическими формами, сохраняя баланс между актуальностью и вечностью. Каждая вещь Maison David создается, чтобы жить долго — сопровождать своего владельца в реальной, настоящей жизни: в работе, в путешествиях, в личных историях. Это не просто гардероб, а состояние уравновешенности и эстетического покоя.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://basket-17.wbcontent.net/vol2778/part277883/277883751/images/big/1.webp,https://basket-17.wbcontent.net/vol2778/part277883/277883751/images/big/2.webp,https://basket-17.wbcontent.net/vol2778/part277883/277883751/images/big/3.webp,https://basket-17.wbcontent.net/vol2778/part277883/277883751/images/big/4.webp,https://basket-17.wbcontent.net/vol2778/part277883/277883751/images/big/5.webp</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Состав: шерсть натуральная 100% | Цвет: серый | Сезон: демисезон | Рост модели на фото: 175 см | Температурный режим: от -5 °C до +10 °C | Покрой: прямой | Воротник: отложной | Тип карманов: прорезные | Особенности модели: Без капюшона, теплый | Пол: Женский | Уход за вещами: Химическая стирка; стирка запрещена; отбеливание запрещено | Комплектация: 1 шт | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>MAISON DAVID</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/528630</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>S, M, L, XS, XL, XXL</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="M2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/288989036/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>288989036</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Короткое шерстяное пальто</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8417</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Черное полупальто женское французского бренда Maison David. Состав: 100% шерсть натуральная. Шерсть отлично согревает, при этом позволяет телу дышать, не создавая парникового эффекта. В шерстяных вещах тепло, но не жарко. Одежда из шерсти — идеальный выбор для зимы и холодного демисезона. Состав подкладки: полиэстер, вискоза.
+Верхняя одежда имеет прямой силуэт. Модель отличает отложной воротник и наличие прорезных карманов. Температурный режим от плюс 10 до минус 5.
+Ухаживайте за вещью правильно, чтобы она дольше служила и радовала вас. Правила по уходу указаны на вшивном ярлычке изделия. Разрешено: химчистка. Запрещено: стирка, отбеливание, глажка, барабанная сушка.
+Полупальто в деловом стиле — удачное решение для офисного гардероба. Это сдержанная элегантность, уверенность и профессионализм. Maison David — дом современной элегантности. Бренд отражает идею французского bon chic, bon genre: искусство быть безупречным без усилий, сочетая гармонию интеллекта и формы, а качество становится главным языком красоты. Бренд соединяет современные тенденции с классическими формами, сохраняя баланс между актуальностью и вечностью. Каждая вещь Maison David создается, чтобы жить долго — сопровождать своего владельца в реальной, настоящей жизни: в работе, в путешествиях, в личных историях. Это не просто гардероб, а состояние уравновешенности и эстетического покоя.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://basket-18.wbcontent.net/vol2889/part288989/288989036/images/big/1.webp,https://basket-18.wbcontent.net/vol2889/part288989/288989036/images/big/2.webp,https://basket-18.wbcontent.net/vol2889/part288989/288989036/images/big/3.webp,https://basket-18.wbcontent.net/vol2889/part288989/288989036/images/big/4.webp,https://basket-18.wbcontent.net/vol2889/part288989/288989036/images/big/5.webp</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Состав: шерсть натуральная 100% | Цвет: черный | Сезон: демисезон | Рост модели на фото: 175 см | Температурный режим: от -5 °C до +10 °C | Покрой: прямой | Воротник: отложной | Тип карманов: прорезные | Особенности модели: Без капюшона, теплый | Пол: Женский | Уход за вещами: Химическая стирка; стирка запрещена; отбеливание запрещено | Комплектация: 1 шт | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>MAISON DAVID</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/528630</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>XS, S, M, L, XL, XXL</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>42</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M3" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/292873097/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>292873097</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Короткое шерстяное пальто</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>8030</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Коричневое полупальто женское французского бренда Maison David. Состав: 100% шерсть натуральная. Шерсть отлично согревает, при этом позволяет телу дышать, не создавая парникового эффекта. В шерстяных вещах тепло, но не жарко. Одежда из шерсти — идеальный выбор для зимы и холодного демисезона. Состав подкладки: полиэстер, вискоза.
+Верхняя одежда имеет прямой силуэт. Модель отличает отложной воротник и наличие прорезных карманов. Температурный режим от плюс 10 до минус 5.
+Ухаживайте за вещью правильно, чтобы она дольше служила и радовала вас. Правила по уходу указаны на вшивном ярлычке изделия. Разрешено: химчистка. Запрещено: стирка, отбеливание, глажка, барабанная сушка.
+Полупальто в стиле кэжуал — удачное дополнение повседневного гардероба. Одежда в стиле кэжуал станет частью ваших комфортных образов на каждый день для работы и отдыха. Maison David — дом современной элегантности. Бренд отражает идею французского bon chic, bon genre: искусство быть безупречным без усилий, сочетая гармонию интеллекта и формы, а качество становится главным языком красоты. Бренд соединяет современные тенденции с классическими формами, сохраняя баланс между актуальностью и вечностью. Каждая вещь Maison David создается, чтобы жить долго — сопровождать своего владельца в реальной, настоящей жизни: в работе, в путешествиях, в личных историях. Это не просто гардероб, а состояние уравновешенности и эстетического покоя.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://basket-18.wbcontent.net/vol2928/part292873/292873097/images/big/1.webp,https://basket-18.wbcontent.net/vol2928/part292873/292873097/images/big/2.webp,https://basket-18.wbcontent.net/vol2928/part292873/292873097/images/big/3.webp,https://basket-18.wbcontent.net/vol2928/part292873/292873097/images/big/4.webp,https://basket-18.wbcontent.net/vol2928/part292873/292873097/images/big/5.webp,https://basket-18.wbcontent.net/vol2928/part292873/292873097/images/big/6.webp</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Состав: шерсть натуральная 100% | Цвет: серо-коричневый | Сезон: демисезон | Рост модели на фото: 175 см | Температурный режим: от -5 °C до +10 °C | Покрой: прямой | Воротник: отложной | Тип карманов: прорезные | Особенности модели: Без капюшона, теплый | Пол: Женский | Уход за вещами: Химическая стирка; стирка запрещена; отбеливание запрещено | Комплектация: 1 шт | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>MAISON DAVID</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/528630</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>XS, S, M, L, XL, XXL</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>27</v>
+      </c>
+      <c r="L4" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M4" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/146055032/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>146055032</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Пальто мужское длинное демисезонное оверсайз синее</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5163</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Пальто мужское длинное синего цвета — это элегантная верхняя одежда для мужчин, юношей, подростков, которые ценят классический стиль и комфорт. Пальто мужское демисезонное утепленное выполнено из натуральной драповой ткани с добавлением шерсти, полиэстера и вискозы, с мягким подкладом с утеплителем ворсовым, что делает его тёплым, уютным и удобным для холодного периода времени года. Пальто мужское универсально: его можно носить зимой, в прохладную осень и ранней весной, сочетая с деловыми или кэжуал, спортивными, фэшн-образами.
+Пальто прямого кроя и удлиненной длины, с аккуратными плечами и широкими рукавами с разрезами по бокам и шлицей. Воротник-стойка с лацканами придаёт строгий стиль и классический акцент, а пуговицы делают образ завершённым и элегантным. Пальто мужское оверсайз свободно садится по фигуре и подходит для мужиков, парней, высоких, невысоких и больших размеров.
+Пальто мужское осеннее легко впишется в любой гардероб. Пальто мужское классическое, базовое, однотонное подчёркивает офисный, рабочий, школьный деловой стиль и гармонично сочетается с модным casual-образом с элементами евростиля. Такое брендовое дизайнерское решение уместно для офиса, учёбы, школы, студентов, прогулок, а в качестве праздничного, нарядного подарка молодежное пальто для мальчика, парня и мужа станет стильным и практичным выбором, находкой стилистов.
+Пальто мужское соединяет классику и современные тренды. Пальто мужское шерстяное отлично сохраняет тепло и форму, делает изделие долговечным, современный силуэт полупальто добавляет актуальности с вставками, карманами, фактурной тканью с ворсом. Качество пошива и подкладки подчёркивает премиальность бренда.
+Мужское пальто однобортное подойдёт для деловых встреч, работы, торжественных случаев, праздников и повседневной носки. Универсальное пальто, которое подчеркнёт индивидуальность, добавит образу уверенности и стиля, а главное — будет радовать многие сезоны.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/1.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/2.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/3.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/4.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/5.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/6.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/7.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/8.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/9.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/10.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/11.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/12.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/13.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/14.webp,https://basket-10.wbcontent.net/vol1460/part146055/146055032/images/big/15.webp</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Состав: шерсть; полиэстер; шерсть 60% полиэстер 40% | Цвет: синий; темно-синий | Пол: Мужской | Сезон: Демисезон | Вид застежки: пуговицы | Рост модели на фото: 182 см | Параметры модели на фото (ОГ-ОТ-ОБ): 92-88-90 | Размер на модели: 46 | Утеплитель: шерсть | Температурный режим: от -10 °C до +10 °C | Материал подкладки: вискоза; полиэстер | Покрой: оверсайз | Тип карманов: прорезные | Тип рукава: длинные | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: пуговицы; оверсайз; длинное | Особенности модели: классическая модель; дышащий материал; однобортная | Уход за вещами: химическая чистка; химчистка | Комплектация: пальто | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>BYDAY</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/65778</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>170-176/44, 170-176/54, 182-188/44, 182-188/46, 182-188/50, 182-188/52</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>11</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2609</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/107713204/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>107713204</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Пальто демисезонное прямое</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6170</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Женское пальто весна-осень.
+Бежевое демисезонное пальто - отличный вариант для тех, кто ищет практичность, удобство и стиль. Эко-шуба с карманами подойдет для любого повседневного образа,а также впишется в любой гардероб делового стиля.  Длина пальто миди позволяет носить его как с платьем, так и с джинсами или брюками.
+Модель выполнена из высококачественного эко-меха. Теплая шерстяная ткань придаст ощущение уюта и комфорта весной или осенью. При изготовлении пальто использовались только премиум-ткани и высококачественная фурнитура. Отстрочка по всему изделию добавляет изюминки в классический стиль. 
+Женская верхняя одежда - показатель вкуса и стиля. Модное демисезонное пальто станет незаменимой вещью в гардеробе.
+Модель прямого кроя создает oversize эффект, поэтому подходит для беременных женщин. Пальто больших размеров. Застежка на кнопки, воротник стойка и карманы - удобство в каждой детали.
+Классический вариант женского полупальто придаст вашему образу стиля и лаконичности. При этом за счет воротника стойки , который застёгивается до конца, спасет от ветра и непогоды. Температурный режим от-5 до +10.
+</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/1.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/2.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/3.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/4.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/5.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/6.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/7.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/8.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/9.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/10.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/11.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/12.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/13.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/14.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/15.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/16.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/17.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/18.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/19.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/20.webp,https://basket-07.wbcontent.net/vol1077/part107713/107713204/images/big/21.webp</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Состав: 64% шерсть, 26% акрил, 7% вискоза, 3% полиэстер | Цвет: бежевый; бежевый лайт; бежевый нейтральный; ванильно-бежевый; светло-бежевый | Пол: Женский | Сезон: Демисезон | Вид застежки: кнопки; Пришивные кнопки | Рост модели на фото: 170 см | Параметры модели на фото (ОГ-ОТ-ОБ): 88-63-95 | Размер на модели: 42 | Утеплитель: без утепления | Температурный режим: -5-+10 | Материал подкладки: полиэстер; вискоза; высококачественный полиэстер | Покрой: прямой | Тип карманов: прорезные | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: без элементов | Особенности модели: Больше размеры для беременных модная модель | Уход за вещами: деликатная химическая чистка; допускается отпаривание | Комплектация: полупальто; вешалка; пакет | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>5 LOVE</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/705312</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>44, 46, 48, 50, 52, 54, 42, 56</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>127</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M6" t="n">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/329473994/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>329473994</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Пальто короткое приталенное весна</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>9445</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Женское пальто Befur – идеальный выбор для прохладной осени и ранней весны.  Модель выполнена из качественной ткани с добавлением натуральной шерсти, что обеспечивает комфорт и приятные тактильные ощущения. Двубортный крой с ветрозащитой надежно защитит от непогоды, а диагональный рисунок придает пальто стильный и современный вид. Прямой крой рукавов и прорезные карманы делают модель удобной в носке. Изготовленное из прочной смеси натуральной шерсти (80%) и полиэстера (20%), оно обеспечит вам комфорт и тепло в осенне-весенний период. Женское  пальто отлично подойдет как на весну, так и на осень и даже на начало зимы! Благодаря своему крою и размерной сетке идеально сядет на высоких и невысоких девушек и на беременных, будущих мам . Удобный пояс при желании легко сделает приталенное пальто. Верхняя одежда хорошо смотрится как со спортивными кроссовками, так и с модными высокими сапогами или с грубыми ботинками.
+Пальто Befur – это сочетание практичности, элегантности и комфорта.
+Обращайте внимание на оригинальный лейбл "Befur" и уникальный QR-код "Честный знак".
+Внимание! Если вам пришло изделие с браком или отсутствует пояс, пожалуйста, скажите сотруднику, что это брак. Так вы поможете нам бороться с недобросовестными покупателями и снизите риск того, что вам придет вещь с браком. 
+</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/1.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/2.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/3.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/4.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/5.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/6.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/7.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/8.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/9.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/10.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/11.webp,https://basket-20.wbcontent.net/vol3294/part329473/329473994/images/big/12.webp</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Состав: натуральная шерсть 80%; полиэстер 20% | Цвет: черный | Пол: Женский | Сезон: демисезон | Вид застежки: пуговицы; кнопки | Рост модели на фото: 165 см | Параметры модели на фото (ОГ-ОТ-ОБ): 83-60-86 | Размер на модели: 42 | Утеплитель: без утеплителя | Температурный режим: от 0 °C до +15 °C | Материал подкладки: вискоза - 70%, п/э - 30% | Покрой: прямой | Тип карманов: прорезные | Тип рукава: Длинный рукав прямого кроя | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: без элементов | Особенности модели: ветрозащита | Уход за вещами: профессиональная химическая чистка в мягком режиме | Комплектация: Пальто - 1 шт; Плечики - 1 шт; Чехол - 1 шт | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Befur</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/367672</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>42, 44, 46, 48, 50</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>79</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M7" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/192213044/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>192213044</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Пальто классическое теплое на весну</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5560</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Пальто Бохо женское из ткани с содержанием натуральной шерсти (80%). Объемный текстильный материал на плотной трикотажной основе, имитирующий натуральный вьющийся мех - ягненка. Фактура на лицевой стороне образует завитки длинной 0,5 см. Сезон весна - осень 2026. Обладает достаточно хорошими теплоизоляционными свойствами, в нем не будет эффекта парника, отлично дышит и отводит влагу ничуть не хуже натурального меха благодаря шерстяным волокнам. Пальто Oversize предполагает свободную, широкую посадку, не стесняющую движения. Такой стиль нужно понимать и любить! Пальто Лёгкое, тёплое и приятное на ощупь станет для Вас хорошим решением на любой случай. Без подклада. До -10, но в холодную погоду его активно используют по верх жилета. Эко шубка,  экошуба, шуба барашек, шуба искусственная.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/1.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/2.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/3.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/4.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/5.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/6.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/7.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/8.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/9.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/10.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/11.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/12.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/13.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/14.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/15.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/16.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/17.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/18.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/19.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/20.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/21.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/22.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/23.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/24.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/25.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/26.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/27.webp,https://basket-13.wbcontent.net/vol1922/part192213/192213044/images/big/28.webp</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Состав: шерсть 80%; Вискоза 20% | Цвет: латте; бежево-розовый; розовый | Пол: Женский | Сезон: Демисезон | Вид застежки: пуговицы | Рост модели на фото: 170 см | Параметры модели на фото (ОГ-ОТ-ОБ): 90-63-93 | Размер на модели: 48-52 | Утеплитель: без утеплителя | Температурный режим: от -10 °C до +15 °C | Материал подкладки: без подкладки | Покрой: прямой | Тип карманов: накладные | Тип рукава: длинные | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: пальто шуба женская зимняя; пальто больших размеров женское; пальто демисезонное женское больших размеров | Особенности модели: шуба чебурашка зимняя большие размеры; одежда на весну; Альпака | Уход за вещами: бережная стирка при 30 градусах; Деликатный отжим без перекручивания | Комплектация: пальто женское шерстяное оверсайз-1 шт; шубка барашек -1шт. | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>milidi</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/61696</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>oversize 54-62</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M8" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/257303252/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>257303252</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Пальто шерстяное демисезонное с воротником стойкой</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>8278</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Окунитесь в стиль и комфорт, выбирая женское пальто для сезона весна-осень. Состав изделия: шерсть - 57%, вискоза - 36%, полиэстер - 7%. Длина пальто по спинке - 63 см. Длина рукава - 63,5 см. Это короткое демисезонное пальто с воротником-стойкой станет вашим верным спутником в любое время года. Однобортное пальто прямого кроя. Воротник-стойка защитит Вас от прохладного ветра, втачные рукава обеспечивают лучшую посадку и комфорт при движении, глубокие карманы с листочкой, отделанные декоративной отстрочкой, придают уникальность, застежкой служат пришивные кнопки. Теплое укороченное пальто привносит в образ изысканность, согреет вас даже в прохладные дни. Дизайнерская вещь подходит для девушек и женщин, ценящих как кэжуал стиль, так и офисную классику. Кофейный-коричневый цвет подойдет к любому образу и станет незаменимой вещью в гардеробе автоледи.
-Кашемировое внимание привлекается длинной линией и модным силуэтом - настоящее утончение 2026 года! Вариации размеров делают изделие доступным даже для подростков и невысоких девочек.
-Будьте уверены: ваше новое ворсовое шерстяное полупальто не только подчеркнет вашу индивидуальность, но и подарит тепло. Смешивайте его с другими модными предметами вашего гардероба – ведь это ключ к созданию стильного ансамбля. Натуральная ткань обеспечивает уют при каждом ношении.
-Ткань имеет ворсистую фактуру, так как в составе большой процент шерсти, из-за этого возможно прилипание волокна, шерсти животных и пыли. Ткань не скатывается, сохраняет цвет и форму. В процессе носки ворс ткани поднимается, поэтому рекомендуем очистить ворс липким роликом, пройтись велюровой щеткой по направлению ворса. Вся продукция бренда КОРЕССИ произведена по высоким стандартам, отшивается на новейшем швейном оборудовании, проходит качественный контроль. Производство Россия. Будем признательны оставленному отзыву! Приятных покупок!
+      <c r="D9" t="n">
+        <v>8541</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Окунитесь в стиль и комфорт, выбирая женское пальто для сезона весна-осень 2026. Длина пальто по спинке - 63 см. Длина рукава - 63,5 см. Это короткое демисезонное пальто с воротником-стойкой станет вашим верным спутником в любое время года. Однобортное пальто прямого кроя. Воротник-стойка защитит Вас от прохладного ветра, втачные рукава обеспечивают лучшую посадку и комфорт при движении, глубокие карманы с листочкой, придают пальто уникальность, застежкой служат пришивные кнопки. Теплое укороченное ворсистое пальто привносит в образ изысканность, согреет вас даже в прохладные дни. Дизайнерская вещь подходит для девушек и женщин, ценящих как кэжуал стиль, так и офисную классику. Бежевый цвет подойдет к любому образу и станет незаменимой вещью в гардеробе автоледи. 
+Кашемировое внимание привлекается длинной линией и модным силуэтом - настоящее утончение 2026 года! Приталенное или оверсайз – выберите то, что подходит именно вам. Вариации размеров делают изделие доступным даже для подростков и невысоких девочек.
+Будьте уверены: ваше новое шерстяное полупальто не только подчеркнет вашу индивидуальность, но и подарит тепло. Смешивайте его с другими модными предметами вашего гардероба – ведь это ключ к созданию стильного ансамбля. Натуральная ворсовая ткань обеспечивает уют при каждом ношении.
+Ткань имеет ворсистую фактуру, так как в составе большой процент шерсти, из-за этого возможно прилипание волокна, шерсти животных и пыли. Ткань не скатывается, сохраняет цвет и форму. В процессе носки ворс ткани поднимается, поэтому рекомендуем очистить ворс липким роликом, пройтись велюровой щеткой по направлению ворса. Вся продукция бренда КОРЕССИ произведена по высоким стандартам, отшивается на новейшем швейном оборудовании, проходит качественный контроль. Производство Россия. Будем признательны оставленному отзыву! Приятных покупок!</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/1.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/2.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/3.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/4.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/5.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/6.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/7.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/8.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/9.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/10.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/11.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/12.webp,https://basket-16.wbcontent.net/vol2573/part257303/257303252/images/big/13.webp</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Состав: шерсть 80%; вискоза 10%; полиэстер 10% | Цвет: бежевый; светло-бежевый | Пол: Женский | Сезон: демисезон | Вид застежки: кнопки | Рост модели на фото: 164 см | Параметры модели на фото (ОГ-ОТ-ОБ): 83-60-89 | Размер на модели: 42 | Утеплитель: без утеплителя | Температурный режим: от 0 °C до +15 °C | Материал подкладки: полиэстер | Покрой: прямой | Тип карманов: прорезные | Тип рукава: длинные | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: застежка на кнопках; глубокие карманы с листочкой; Ворсовая ткань | Особенности модели: однобортная; ветрозащита; износостойкость | Уход за вещами: деликатная химическая чистка; допускается отпаривание | Комплектация: Пальто - 1 шт; Чехол с зип-пакетом или Упаковочная сумка-чемодан | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Coressi</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/26796</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>42, 48, 52</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>10</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="M9" t="n">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/329899819/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>329899819</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Пальто шерстяное демисезонное с воротником стойкой</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>8016</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Окунитесь в стиль и комфорт, выбирая женское пальто для сезона весна-осень 2026. Длина пальто по спинке - 63 см. Длина рукава - 63,5 см. Это короткое демисезонное пальто с воротником-стойкой станет вашим верным спутником в любое время года. Однобортное пальто прямого кроя. Воротник-стойка защитит Вас от прохладного ветра, втачные рукава обеспечивают лучшую посадку и комфорт при движении, глубокие карманы с листочкой, придают пальто уникальность, застежкой служат пришивные кнопки. Теплое укороченное ворсистое пальто привносит в образ изысканность, согреет вас даже в прохладные дни. Дизайнерская вещь подходит для девушек и женщин, ценящих как кэжуал стиль, так и офисную классику. Серый цвет подойдет к любому образу и станет незаменимой вещью в гардеробе автоледи. 
+Кашемировое внимание привлекается длинной линией и модным силуэтом - настоящее утончение 2026 года! Приталенное или оверсайз – выберите то, что подходит именно вам. Вариации размеров делают изделие доступным даже для подростков и невысоких девочек.
+Будьте уверены: ваше новое шерстяное полупальто не только подчеркнет вашу индивидуальность, но и подарит тепло. Смешивайте его с другими модными предметами вашего гардероба – ведь это ключ к созданию стильного ансамбля. Натуральная ворсовая ткань обеспечивает уют при каждом ношении.
+Ткань имеет ворсистую фактуру, так как в составе большой процент шерсти, из-за этого возможно прилипание волокна, шерсти животных и пыли. Ткань не скатывается, сохраняет цвет и форму. В процессе носки ворс ткани поднимается, поэтому рекомендуем очистить ворс липким роликом, пройтись велюровой щеткой по направлению ворса. Вся продукция бренда КОРЕССИ произведена по высоким стандартам, отшивается на новейшем швейном оборудовании, проходит качественный контроль. Производство Россия. Будем признательны оставленному отзыву! Приятных покупок!</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/1.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/2.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/3.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/4.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/5.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/6.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/7.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/8.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/9.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/10.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/11.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/12.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/13.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/14.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/15.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/16.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/17.webp,https://basket-20.wbcontent.net/vol3298/part329899/329899819/images/big/18.webp</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Состав: шерсть 80%; вискоза 10%; полиэстер 10% | Цвет: серый | Пол: Женский | Сезон: демисезон | Вид застежки: кнопки | Рост модели на фото: 164 см | Параметры модели на фото (ОГ-ОТ-ОБ): 83-60-89 | Размер на модели: 42 | Утеплитель: без утеплителя | Температурный режим: от 0 °C до +15 °C | Материал подкладки: полиэстер | Покрой: прямой | Тип карманов: прорезные | Тип рукава: длинные | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: застежка на кнопках; глубокие карманы с листочкой; Ворсовая ткань | Особенности модели: однобортная; ветрозащита; износостойкость | Уход за вещами: деликатная химическая чистка; допускается отпаривание | Комплектация: Пальто - 1 шт; Упаковочная сумка-чемодан | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Coressi</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/26796</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="M10" t="n">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/catalog/197262900/detail.aspx</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>197262900</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Пальто женское демисезонное оверсайз теплое длинное</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>7750</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Пальто демисезонное женское идеально подходит для тех, кто ищет верхнюю одежду, которая будет актуальна как в весенний, так и в осенний период.Это длинная, теплая, демисезонная модель предназначена для женщин, которые ценят стиль и комфорт в верхней одежде. Оно отлично подходит для весенне-осеннего периода, когда погода может быть непредсказуемой. Пальто сочетает в себе элегантный дизайн и функциональность, что делает его универсальным вариантом для повседневного ношения.
+Основное предназначение этой модели — защита от холода и ветра в межсезонье. Оно выполнено из высококачественных шерстяных материалов, что обеспечивает тепло и комфорт даже в прохладные дни. Модель имеет классическую форму, что позволяет легко комбинировать ее с различными нарядами, будь то офисный стиль или повседневный образ.  цвет делает его особенно стильным и универсальным, позволяя сочетать его с разнообразной одеждой. Пояс идет в комплекте. Очень удобные и глубокие карманы. 
+Длинный крой обеспечивает дополнительное тепло, а также создает аккуратный силуэт. Мягкая шерсть в составе материала обеспечивает приятные ощущения при носке. В этом пальто вы будете выглядеть стильно и ощущать себя комфортно в любых условиях.
+Модель отлично подойдет для городских прогулок, деловых встреч или встреч с друзьями. Пальто женское весна-осень легко можно дополнить шарфом или шапкой, что сделает ваш образ завершенным. Оно станет надежным спутником в вашем гардеробе, добавив в него ярких акцентов и создавая множество стильных образов.
 </t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://basket-15.wbcontent.net/vol2398/part239833/239833866/images/big/1.webp,https://basket-15.wbcontent.net/vol2398/part239833/239833866/images/big/2.webp,https://basket-15.wbcontent.net/vol2398/part239833/239833866/images/big/3.webp,https://basket-15.wbcontent.net/vol2398/part239833/239833866/images/big/4.webp,https://basket-15.wbcontent.net/vol2398/part239833/239833866/images/big/5.webp</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Состав: шерсть; вискоза; полиэстер | Цвет: коричневый; кофейный | Пол: Женский | Сезон: Демисезон | Вид застежки: кнопки | Рост модели на фото: 164 см | Параметры модели на фото (ОГ-ОТ-ОБ): 83-60-89 | Размер на модели: 42 | Утеплитель: без утеплителя | Температурный режим: от 0 °C до +15 °C | Материал подкладки: полиэстер | Покрой: прямой | Тип карманов: прорезные | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: декоративная отстрочка; воротник стойка; карманы | Особенности модели: однобортная; ветрозащита; износостойкость | Уход за вещами: деликатная химическая чистка; допускается отпаривание | Комплектация: Пальто - 1 шт; Упаковочная сумка-чемодан | Страна производства: Россия</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Coressi</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>https://www.wildberries.ru/seller/26796</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>42, 44, 46, 48, 50, 52, 54</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>166</v>
-      </c>
-      <c r="L2" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1840</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/1.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/2.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/3.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/4.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/5.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/6.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/7.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/8.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/9.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/10.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/11.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/12.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/13.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/14.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/15.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/16.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/17.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/18.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/19.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/20.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/21.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/22.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/23.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/24.webp,https://basket-13.wbcontent.net/vol1972/part197262/197262900/images/big/25.webp</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Состав: 50% шерсть, 30% вискоза, 20% поливискоза | Цвет: серый; натуральный серый; зернистый светло-серый | Пол: Женский | Сезон: демисезон | Вид застежки: пуговицы; супатная | Рост модели на фото: 177 см | Параметры модели на фото (ОГ-ОТ-ОБ): 86-64-93 | Размер на модели: 46 | Утеплитель: без утеплителя | Температурный режим: от +3 до +15 | Материал подкладки: полиэстер | Покрой: оверсайз | Тип карманов: накладные | Тип рукава: длинные | Опции капюшона: без капюшона | Опции опушки: без опушки | Декоративные элементы: карманы | Особенности модели: ветрозащита | Уход за вещами: допускается отпаривание; деликатная химическая чистка | Комплектация: пояс; пальто | Страна производства: Россия</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EURYDIKE</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://www.wildberries.ru/seller/3971567</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>42, 44, 46, 48, 50, 52</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>22</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M11" t="n">
+        <v>508</v>
       </c>
     </row>
   </sheetData>

</xml_diff>